<commit_message>
Update test file for SavingTests.DeletingAllPicturesRemovesDrawingPart. No semantic change, styles part was written with a new writer.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Other/Drawings/NoDrawings/outputfile.xlsx
+++ b/ClosedXML.Tests/Resource/Other/Drawings/NoDrawings/outputfile.xlsx
@@ -48,15 +48,16 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>

</xml_diff>